<commit_message>
feat: add GRC routes, standard enablement controller, and service
</commit_message>
<xml_diff>
--- a/grc_wisdom_api/scripts/verify/_tmp_reports/Annual_plan.xlsx
+++ b/grc_wisdom_api/scripts/verify/_tmp_reports/Annual_plan.xlsx
@@ -12,20 +12,23 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="63">
   <si>
     <t>Annual Audit Plan</t>
   </si>
   <si>
+    <t>OmniOps</t>
+  </si>
+  <si>
+    <t>CONFIDENTIAL</t>
+  </si>
+  <si>
     <t>2026 Internal Audit Plan (2026) — Approved</t>
   </si>
   <si>
     <t>Organisation</t>
   </si>
   <si>
-    <t>OmniOps</t>
-  </si>
-  <si>
     <t>Engagement</t>
   </si>
   <si>
@@ -38,7 +41,7 @@
     <t>Generated at</t>
   </si>
   <si>
-    <t>2026-08-17 15:43 UTC</t>
+    <t>2026-09-23 10:59 UTC</t>
   </si>
   <si>
     <t>Visibility</t>
@@ -47,6 +50,12 @@
     <t>SUBTREE</t>
   </si>
   <si>
+    <t>Document reference</t>
+  </si>
+  <si>
+    <t>1906-20260923105958</t>
+  </si>
+  <si>
     <t>Quarter</t>
   </si>
   <si>
@@ -92,7 +101,7 @@
     <t>100</t>
   </si>
   <si>
-    <t>Mahmoud Abdulaziz</t>
+    <t>Mehdi Tantaoui</t>
   </si>
   <si>
     <t>Planned</t>
@@ -101,6 +110,15 @@
     <t>Risk tier Medium (score 3.45).</t>
   </si>
   <si>
+    <t>Procure to pay</t>
+  </si>
+  <si>
+    <t>3.85</t>
+  </si>
+  <si>
+    <t>Risk tier Medium (score 3.85).</t>
+  </si>
+  <si>
     <t>Third-party and cloud management</t>
   </si>
   <si>
@@ -119,18 +137,18 @@
     <t>Risk tier High (score 4.95). Never audited.</t>
   </si>
   <si>
-    <t>Procure to pay</t>
-  </si>
-  <si>
-    <t>3.85</t>
-  </si>
-  <si>
-    <t>Risk tier Medium (score 3.85).</t>
-  </si>
-  <si>
     <t>Q2</t>
   </si>
   <si>
+    <t>Treasury and cash management</t>
+  </si>
+  <si>
+    <t>3.83</t>
+  </si>
+  <si>
+    <t>Risk tier Medium (score 3.83).</t>
+  </si>
+  <si>
     <t>Personal data processing</t>
   </si>
   <si>
@@ -140,15 +158,6 @@
     <t>Risk tier High (score 4.5). Never audited.</t>
   </si>
   <si>
-    <t>Treasury and cash management</t>
-  </si>
-  <si>
-    <t>3.83</t>
-  </si>
-  <si>
-    <t>Risk tier Medium (score 3.83).</t>
-  </si>
-  <si>
     <t>Q3</t>
   </si>
   <si>
@@ -173,6 +182,18 @@
     <t>Q4</t>
   </si>
   <si>
+    <t>Core banking platform</t>
+  </si>
+  <si>
+    <t>System</t>
+  </si>
+  <si>
+    <t>4.3</t>
+  </si>
+  <si>
+    <t>Risk tier High (score 4.3).</t>
+  </si>
+  <si>
     <t>Payroll and HR operations</t>
   </si>
   <si>
@@ -180,25 +201,13 @@
   </si>
   <si>
     <t>Risk tier Medium (score 3.5).</t>
-  </si>
-  <si>
-    <t>Core banking platform</t>
-  </si>
-  <si>
-    <t>System</t>
-  </si>
-  <si>
-    <t>4.3</t>
-  </si>
-  <si>
-    <t>Risk tier High (score 4.3).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -210,6 +219,16 @@
       <b/>
       <color rgb="FF0B1524"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0F7A5A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF646F85"/>
+      <sz val="9"/>
     </font>
     <font>
       <color rgb="FF646F85"/>
@@ -226,7 +245,7 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF0B1524"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -239,7 +258,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF5F7FA"/>
+        <fgColor rgb="FF0F7A5A"/>
       </patternFill>
     </fill>
   </fills>
@@ -273,16 +292,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -630,7 +651,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -647,44 +668,62 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+    <row r="3" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+    </row>
+    <row r="4" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B6" s="6" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B7" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="B8" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="4" t="s">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="B9" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="4" t="s">
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
         <v>10</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -708,294 +747,294 @@
     <col min="9" max="9" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" s="6" t="s">
+    <row r="1" ht="22" customHeight="1" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="B1" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="C1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="D1" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="E1" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="F1" s="8" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+      <c r="G1" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="H1" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="I1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D2" s="8" t="s">
+    </row>
+    <row r="2" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="B2" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="C2" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="D2" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="E2" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="F2" s="10" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" s="8" t="s">
+      <c r="G2" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="H2" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="I2" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="E3" s="8" t="s">
+    </row>
+    <row r="3" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="C3" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="G3" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="H3" s="8" t="s">
+      <c r="E3" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="F3" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="I3" s="10" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="8" t="s">
+    <row r="4" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C4" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" s="8" t="s">
+      <c r="C4" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="E4" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4" s="8" t="s">
+      <c r="D4" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="G4" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" s="8" t="s">
+      <c r="D5" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="E5" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="I4" s="8" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="F5" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="F6" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="H5" s="8" t="s">
+      <c r="G6" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="I5" s="8" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+      <c r="F7" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E8" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="F6" s="8" t="s">
+      <c r="F8" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="I8" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="I9" s="10" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="G6" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="H6" s="8" t="s">
+      <c r="D10" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="E10" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="I6" s="8" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="I7" s="8" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="I8" s="8" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="H9" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="I9" s="8" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="I10" s="8" t="s">
-        <v>59</v>
+      <c r="F10" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10" s="10" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>